<commit_message>
docs(testing): narrow SCRUM-34's read-only rule to rejected requests
The story locks only what its acceptance criteria ask (a rejected request
is read-only for its Organiser) and changes only its own code, so
TC_E03S03_11 no longer covers completed events or Coordinators.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 011026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 011026.xlsx
@@ -4344,33 +4344,30 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Verify that a completed or rejected request cannot be edited by its Organiser or Coordinator</t>
+          <t>Verify that an Event Organiser cannot edit their rejected request</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Event EVT-2004 has status "Completed", was submitted by organiser_a@clienta.com and is assigned to coord_a@connectsphere.com. Event EVT-3005 has status "Rejected" and was submitted by organiser_b@clienta.com</t>
+          <t>Event EVT-3005 has status "Rejected" and was submitted by organiser_b@clienta.com</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>1. Sign in as organiser_a@clienta.com
- 2. Attempt to change the title of EVT-2004 to "EVT-2004 Renamed"
- 3. Sign in as coord_a@connectsphere.com
- 4. Attempt to change the expected attendance of EVT-2004 to 60
- 5. Sign in as organiser_b@clienta.com
- 6. Attempt to change the description of EVT-3005
- 7. Re-read EVT-2004 and EVT-3005</t>
+          <t>1. Sign in as organiser_b@clienta.com
+ 2. Attempt to change the title of EVT-3005 to "EVT-3005 Budget Review (revised)"
+ 3. Attempt to change the description of EVT-3005
+ 4. Re-read EVT-3005</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Events: EVT-2004 (Completed), EVT-3005 (Rejected) · New title: "EVT-2004 Renamed" · New expected attendance: 60</t>
+          <t>Event: EVT-3005 (Rejected) · New title: "EVT-3005 Budget Review (revised)"</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>All three edits are refused with a message that the request is completed or rejected and can no longer be changed. Neither event's fields change. A cancelled request is refused the same way (covered by the backend test, as the seeded data has no cancelled event)</t>
+          <t>Both edits are refused with a message that the request is rejected and can no longer be changed, with no offer to raise a change request. EVT-3005's title and description are unchanged, and it stays "Rejected"</t>
         </is>
       </c>
     </row>

</xml_diff>